<commit_message>
Login and Manage Page done
</commit_message>
<xml_diff>
--- a/tests/projectWorkSpaceERP/HCM/CoreHR/HireAnEmployeeTestData.xlsx
+++ b/tests/projectWorkSpaceERP/HCM/CoreHR/HireAnEmployeeTestData.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="58">
   <si>
     <t>Dataset</t>
   </si>
@@ -28,6 +28,9 @@
     <t>Password</t>
   </si>
   <si>
+    <t>bypasscode</t>
+  </si>
+  <si>
     <t>Book</t>
   </si>
   <si>
@@ -136,22 +139,16 @@
     <t>True</t>
   </si>
   <si>
-    <t>16-Jan-2025</t>
-  </si>
-  <si>
     <t>Hire to fill vacant position</t>
   </si>
   <si>
     <t>Hire</t>
   </si>
   <si>
-    <t>Arvinmeritor Technology, LLC</t>
+    <t>D00 TCS US LE</t>
   </si>
   <si>
     <t>Male</t>
-  </si>
-  <si>
-    <t>06-Jan-1988</t>
   </si>
   <si>
     <t>Home Fax</t>
@@ -198,7 +195,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -209,12 +206,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -246,7 +237,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -257,16 +248,16 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -280,9 +271,6 @@
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -586,31 +574,31 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AH8"/>
+  <dimension ref="A1:AI8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="8" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="8" width="19.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="8" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="8" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="8" width="19.14785714285714" customWidth="1" bestFit="1"/>
     <col min="9" max="9" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="10" max="10" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="11" max="11" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="13" max="13" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="8" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="8" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="18" max="18" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="21" max="21" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="23" max="23" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="24" max="24" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="25" max="25" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
@@ -620,9 +608,10 @@
     <col min="29" max="29" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="30" max="30" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="31" max="31" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="32" max="32" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="33" max="33" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="34" max="34" style="10" width="15.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="33" max="33" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="34" max="34" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="35" max="35" style="10" width="15.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
@@ -659,13 +648,13 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
       <c r="O1" s="1" t="s">
@@ -674,22 +663,22 @@
       <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
       <c r="R1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
       <c r="U1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="3" t="s">
         <v>21</v>
       </c>
       <c r="W1" s="1" t="s">
@@ -719,31 +708,34 @@
       <c r="AE1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="4" t="s">
+      <c r="AF1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AG1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="2" t="s">
+      <c r="AH1" s="1" t="s">
         <v>33</v>
+      </c>
+      <c r="AI1" s="2" t="s">
+        <v>34</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="20.25">
       <c r="A2" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E2" s="1" t="s">
         <v>38</v>
+      </c>
+      <c r="E2" s="4">
+        <v>380871860776</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>39</v>
@@ -751,86 +743,89 @@
       <c r="G2" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="5">
+        <v>46023</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="M2" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="N2" s="1" t="s">
+      <c r="L2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="N2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="O2" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="P2" s="5">
+        <v>30683</v>
+      </c>
+      <c r="Q2" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="R2" s="7">
+        <v>212</v>
+      </c>
+      <c r="S2" s="7">
+        <v>7123813</v>
+      </c>
+      <c r="T2" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="Q2" s="6">
-        <v>212</v>
-      </c>
-      <c r="R2" s="6">
-        <v>7123813</v>
-      </c>
-      <c r="S2" s="1" t="s">
+      <c r="U2" s="7">
+        <v>123</v>
+      </c>
+      <c r="V2" s="7">
+        <v>21225</v>
+      </c>
+      <c r="W2" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="T2" s="6">
-        <v>123</v>
-      </c>
-      <c r="U2" s="6">
-        <v>21225</v>
-      </c>
-      <c r="V2" s="1" t="s">
+      <c r="X2" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="Y2" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="X2" s="1" t="s">
+      <c r="Z2" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="Y2" s="1" t="s">
+      <c r="AA2" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="Z2" s="1" t="s">
+      <c r="AB2" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="AA2" s="1" t="s">
+      <c r="AC2" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="AB2" s="1" t="s">
+      <c r="AD2" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="AC2" s="1" t="s">
+      <c r="AE2" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="AD2" s="1" t="s">
+      <c r="AF2" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="AE2" s="1" t="s">
+      <c r="AG2" s="7">
+        <v>4000</v>
+      </c>
+      <c r="AH2" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="AF2" s="6">
-        <v>4000</v>
-      </c>
-      <c r="AG2" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="AH2" s="5" t="s">
-        <v>49</v>
+      <c r="AI2" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="20.25">
@@ -842,20 +837,20 @@
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="3"/>
       <c r="K3" s="1"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
       <c r="O3" s="1"/>
       <c r="P3" s="1"/>
-      <c r="Q3" s="6"/>
-      <c r="R3" s="6"/>
-      <c r="S3" s="1"/>
-      <c r="T3" s="6"/>
-      <c r="U3" s="6"/>
-      <c r="V3" s="1"/>
+      <c r="Q3" s="1"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="1"/>
+      <c r="U3" s="7"/>
+      <c r="V3" s="7"/>
       <c r="W3" s="1"/>
       <c r="X3" s="1"/>
       <c r="Y3" s="1"/>
@@ -865,9 +860,10 @@
       <c r="AC3" s="1"/>
       <c r="AD3" s="1"/>
       <c r="AE3" s="1"/>
-      <c r="AF3" s="7"/>
-      <c r="AG3" s="1"/>
-      <c r="AH3" s="6"/>
+      <c r="AF3" s="1"/>
+      <c r="AG3" s="7"/>
+      <c r="AH3" s="1"/>
+      <c r="AI3" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="20.25">
       <c r="A4" s="1"/>
@@ -881,17 +877,17 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
       <c r="O4" s="1"/>
       <c r="P4" s="1"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
-      <c r="S4" s="1"/>
-      <c r="T4" s="6"/>
-      <c r="U4" s="6"/>
-      <c r="V4" s="1"/>
+      <c r="Q4" s="1"/>
+      <c r="R4" s="7"/>
+      <c r="S4" s="7"/>
+      <c r="T4" s="1"/>
+      <c r="U4" s="7"/>
+      <c r="V4" s="7"/>
       <c r="W4" s="1"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="1"/>
@@ -901,12 +897,13 @@
       <c r="AC4" s="1"/>
       <c r="AD4" s="1"/>
       <c r="AE4" s="1"/>
-      <c r="AF4" s="7"/>
-      <c r="AG4" s="1"/>
-      <c r="AH4" s="6"/>
+      <c r="AF4" s="1"/>
+      <c r="AG4" s="7"/>
+      <c r="AH4" s="1"/>
+      <c r="AI4" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="20.25">
-      <c r="A5" s="5"/>
+      <c r="A5" s="6"/>
       <c r="B5" s="1"/>
       <c r="C5" s="3"/>
       <c r="D5" s="1"/>
@@ -917,17 +914,17 @@
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="3"/>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
-      <c r="Q5" s="6"/>
-      <c r="R5" s="6"/>
-      <c r="S5" s="1"/>
-      <c r="T5" s="6"/>
-      <c r="U5" s="6"/>
-      <c r="V5" s="1"/>
+      <c r="Q5" s="1"/>
+      <c r="R5" s="7"/>
+      <c r="S5" s="7"/>
+      <c r="T5" s="1"/>
+      <c r="U5" s="7"/>
+      <c r="V5" s="7"/>
       <c r="W5" s="1"/>
       <c r="X5" s="1"/>
       <c r="Y5" s="1"/>
@@ -937,9 +934,10 @@
       <c r="AC5" s="1"/>
       <c r="AD5" s="1"/>
       <c r="AE5" s="1"/>
-      <c r="AF5" s="7"/>
-      <c r="AG5" s="1"/>
-      <c r="AH5" s="6"/>
+      <c r="AF5" s="1"/>
+      <c r="AG5" s="7"/>
+      <c r="AH5" s="1"/>
+      <c r="AI5" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="20.25">
       <c r="A6" s="1"/>
@@ -951,19 +949,19 @@
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
-      <c r="N6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
-      <c r="Q6" s="6"/>
-      <c r="R6" s="6"/>
-      <c r="S6" s="1"/>
-      <c r="T6" s="6"/>
-      <c r="U6" s="6"/>
-      <c r="V6" s="1"/>
+      <c r="Q6" s="1"/>
+      <c r="R6" s="7"/>
+      <c r="S6" s="7"/>
+      <c r="T6" s="1"/>
+      <c r="U6" s="7"/>
+      <c r="V6" s="7"/>
       <c r="W6" s="1"/>
       <c r="X6" s="1"/>
       <c r="Y6" s="1"/>
@@ -973,9 +971,10 @@
       <c r="AC6" s="1"/>
       <c r="AD6" s="1"/>
       <c r="AE6" s="1"/>
-      <c r="AF6" s="7"/>
-      <c r="AG6" s="1"/>
-      <c r="AH6" s="6"/>
+      <c r="AF6" s="1"/>
+      <c r="AG6" s="7"/>
+      <c r="AH6" s="1"/>
+      <c r="AI6" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="20.25">
       <c r="A7" s="1"/>
@@ -989,17 +988,17 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
-      <c r="N7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
       <c r="O7" s="1"/>
       <c r="P7" s="1"/>
-      <c r="Q7" s="6"/>
-      <c r="R7" s="6"/>
-      <c r="S7" s="1"/>
-      <c r="T7" s="6"/>
-      <c r="U7" s="6"/>
-      <c r="V7" s="1"/>
+      <c r="Q7" s="1"/>
+      <c r="R7" s="7"/>
+      <c r="S7" s="7"/>
+      <c r="T7" s="1"/>
+      <c r="U7" s="7"/>
+      <c r="V7" s="7"/>
       <c r="W7" s="1"/>
       <c r="X7" s="1"/>
       <c r="Y7" s="1"/>
@@ -1009,9 +1008,10 @@
       <c r="AC7" s="1"/>
       <c r="AD7" s="1"/>
       <c r="AE7" s="1"/>
-      <c r="AF7" s="7"/>
-      <c r="AG7" s="1"/>
-      <c r="AH7" s="6"/>
+      <c r="AF7" s="1"/>
+      <c r="AG7" s="7"/>
+      <c r="AH7" s="1"/>
+      <c r="AI7" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="20.25">
       <c r="A8" s="1"/>
@@ -1025,17 +1025,17 @@
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
-      <c r="N8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
-      <c r="Q8" s="6"/>
-      <c r="R8" s="6"/>
-      <c r="S8" s="1"/>
-      <c r="T8" s="6"/>
-      <c r="U8" s="6"/>
-      <c r="V8" s="1"/>
+      <c r="Q8" s="1"/>
+      <c r="R8" s="7"/>
+      <c r="S8" s="7"/>
+      <c r="T8" s="1"/>
+      <c r="U8" s="7"/>
+      <c r="V8" s="7"/>
       <c r="W8" s="1"/>
       <c r="X8" s="1"/>
       <c r="Y8" s="1"/>
@@ -1045,9 +1045,10 @@
       <c r="AC8" s="1"/>
       <c r="AD8" s="1"/>
       <c r="AE8" s="1"/>
-      <c r="AF8" s="7"/>
-      <c r="AG8" s="1"/>
-      <c r="AH8" s="6"/>
+      <c r="AF8" s="1"/>
+      <c r="AG8" s="7"/>
+      <c r="AH8" s="1"/>
+      <c r="AI8" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Hire an Employee Pass
</commit_message>
<xml_diff>
--- a/tests/projectWorkSpaceERP/HCM/CoreHR/HireAnEmployeeTestData.xlsx
+++ b/tests/projectWorkSpaceERP/HCM/CoreHR/HireAnEmployeeTestData.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="49">
   <si>
     <t>Dataset</t>
   </si>
@@ -31,9 +31,6 @@
     <t>bypasscode</t>
   </si>
   <si>
-    <t>Book</t>
-  </si>
-  <si>
     <t>PersonalDetails</t>
   </si>
   <si>
@@ -79,7 +76,7 @@
     <t>AddressLine1</t>
   </si>
   <si>
-    <t>ZIPCode</t>
+    <t>City</t>
   </si>
   <si>
     <t>MaritalStatus</t>
@@ -97,7 +94,7 @@
     <t>Grade</t>
   </si>
   <si>
-    <t>CumminsAssignmentStatus</t>
+    <t>AssignmentStatus</t>
   </si>
   <si>
     <t>Location</t>
@@ -133,21 +130,15 @@
     <t>@+34Ll8I_|ib</t>
   </si>
   <si>
-    <t>US Corp</t>
-  </si>
-  <si>
     <t>True</t>
   </si>
   <si>
-    <t>Hire to fill vacant position</t>
+    <t>Retal Legal Entity</t>
   </si>
   <si>
     <t>Hire</t>
   </si>
   <si>
-    <t>D00 TCS US LE</t>
-  </si>
-  <si>
     <t>Male</t>
   </si>
   <si>
@@ -157,19 +148,19 @@
     <t>Mailing Address</t>
   </si>
   <si>
+    <t>Riyadh</t>
+  </si>
+  <si>
+    <t>RETAL KHOBAR BU</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>D00 TCS US Business unit</t>
-  </si>
-  <si>
-    <t>Annual Salary</t>
-  </si>
-  <si>
-    <t>False</t>
-  </si>
-  <si>
-    <t>United States</t>
+    <t>false</t>
+  </si>
+  <si>
+    <t>Saudi Arabia</t>
   </si>
 </sst>
 </file>
@@ -233,29 +224,29 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -577,7 +568,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AI8"/>
+  <dimension ref="A1:AH8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
@@ -585,23 +576,23 @@
     <col min="3" max="3" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="13" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="11" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="14" width="19.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="11" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="14" width="19.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="9" max="9" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="10" max="10" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="11" max="11" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="15" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="13" max="13" style="15" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="15" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="14" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="14" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="16" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="18" max="18" style="16" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="16" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="16" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="16" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="16" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="15" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="23" max="23" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="24" max="24" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="25" max="25" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
@@ -611,10 +602,9 @@
     <col min="29" max="29" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="30" max="30" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="31" max="31" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="32" max="32" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="33" max="33" style="16" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="34" max="34" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="35" max="35" style="15" width="15.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="16" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="33" max="33" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="34" max="34" style="15" width="15.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
@@ -636,10 +626,10 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
@@ -651,37 +641,37 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="5" t="s">
         <v>16</v>
       </c>
       <c r="R1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="5" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
       <c r="W1" s="1" t="s">
@@ -711,122 +701,100 @@
       <c r="AE1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AF1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="5" t="s">
+      <c r="AG1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AH1" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="AI1" s="2" t="s">
-        <v>34</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="20.25">
       <c r="A2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>38</v>
       </c>
       <c r="E2" s="6">
         <v>380871860776</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G2" s="7">
+        <v>46023</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H2" s="7">
-        <v>46023</v>
-      </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M2" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="N2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="O2" s="7">
+        <v>30683</v>
+      </c>
+      <c r="P2" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="Q2" s="6">
+        <v>212</v>
+      </c>
+      <c r="R2" s="6">
+        <v>7123813</v>
+      </c>
+      <c r="S2" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="L2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="N2" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="O2" s="1" t="s">
+      <c r="T2" s="6">
+        <v>123</v>
+      </c>
+      <c r="U2" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="P2" s="7">
-        <v>30683</v>
-      </c>
-      <c r="Q2" s="1" t="s">
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="R2" s="9">
-        <v>212</v>
-      </c>
-      <c r="S2" s="9">
-        <v>7123813</v>
-      </c>
-      <c r="T2" s="1" t="s">
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+      <c r="AC2" s="1"/>
+      <c r="AD2" s="1"/>
+      <c r="AE2" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="U2" s="9">
-        <v>123</v>
-      </c>
-      <c r="V2" s="9"/>
-      <c r="W2" s="10" t="s">
+      <c r="AF2" s="6"/>
+      <c r="AG2" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="X2" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="Y2" s="1" t="s">
+      <c r="AH2" s="8" t="s">
         <v>48</v>
-      </c>
-      <c r="Z2" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="AA2" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="AB2" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="AC2" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="AD2" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="AE2" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="AF2" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="AG2" s="9">
-        <v>4000</v>
-      </c>
-      <c r="AH2" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AI2" s="8" t="s">
-        <v>51</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="20.25">
@@ -834,24 +802,24 @@
       <c r="B3" s="1"/>
       <c r="C3" s="5"/>
       <c r="D3" s="1"/>
-      <c r="E3" s="3"/>
+      <c r="E3" s="10"/>
       <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="5"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="1"/>
       <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="9"/>
-      <c r="N3" s="9"/>
-      <c r="O3" s="1"/>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="1"/>
-      <c r="R3" s="9"/>
-      <c r="S3" s="9"/>
-      <c r="T3" s="1"/>
-      <c r="U3" s="9"/>
-      <c r="V3" s="9"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6"/>
+      <c r="S3" s="1"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="1"/>
       <c r="W3" s="1"/>
       <c r="X3" s="1"/>
       <c r="Y3" s="1"/>
@@ -861,34 +829,33 @@
       <c r="AC3" s="1"/>
       <c r="AD3" s="1"/>
       <c r="AE3" s="1"/>
-      <c r="AF3" s="1"/>
-      <c r="AG3" s="9"/>
-      <c r="AH3" s="1"/>
-      <c r="AI3" s="9"/>
+      <c r="AF3" s="6"/>
+      <c r="AG3" s="1"/>
+      <c r="AH3" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="20.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="5"/>
       <c r="D4" s="2"/>
-      <c r="E4" s="3"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
-      <c r="O4" s="1"/>
-      <c r="P4" s="4"/>
-      <c r="Q4" s="1"/>
-      <c r="R4" s="9"/>
-      <c r="S4" s="9"/>
-      <c r="T4" s="1"/>
-      <c r="U4" s="9"/>
-      <c r="V4" s="9"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="6"/>
+      <c r="U4" s="6"/>
+      <c r="V4" s="1"/>
       <c r="W4" s="1"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="1"/>
@@ -898,34 +865,33 @@
       <c r="AC4" s="1"/>
       <c r="AD4" s="1"/>
       <c r="AE4" s="1"/>
-      <c r="AF4" s="1"/>
-      <c r="AG4" s="9"/>
-      <c r="AH4" s="1"/>
-      <c r="AI4" s="9"/>
+      <c r="AF4" s="6"/>
+      <c r="AG4" s="1"/>
+      <c r="AH4" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="20.25">
       <c r="A5" s="8"/>
       <c r="B5" s="1"/>
       <c r="C5" s="5"/>
       <c r="D5" s="1"/>
-      <c r="E5" s="3"/>
+      <c r="E5" s="10"/>
       <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="9"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="4"/>
-      <c r="Q5" s="1"/>
-      <c r="R5" s="9"/>
-      <c r="S5" s="9"/>
-      <c r="T5" s="1"/>
-      <c r="U5" s="9"/>
-      <c r="V5" s="9"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="1"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="1"/>
+      <c r="T5" s="6"/>
+      <c r="U5" s="6"/>
+      <c r="V5" s="1"/>
       <c r="W5" s="1"/>
       <c r="X5" s="1"/>
       <c r="Y5" s="1"/>
@@ -935,34 +901,33 @@
       <c r="AC5" s="1"/>
       <c r="AD5" s="1"/>
       <c r="AE5" s="1"/>
-      <c r="AF5" s="1"/>
-      <c r="AG5" s="9"/>
-      <c r="AH5" s="1"/>
-      <c r="AI5" s="9"/>
+      <c r="AF5" s="6"/>
+      <c r="AG5" s="1"/>
+      <c r="AH5" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="20.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="5"/>
       <c r="D6" s="1"/>
-      <c r="E6" s="3"/>
+      <c r="E6" s="10"/>
       <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="1"/>
       <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="1"/>
-      <c r="P6" s="4"/>
-      <c r="Q6" s="1"/>
-      <c r="R6" s="9"/>
-      <c r="S6" s="9"/>
-      <c r="T6" s="1"/>
-      <c r="U6" s="9"/>
-      <c r="V6" s="9"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="1"/>
+      <c r="T6" s="6"/>
+      <c r="U6" s="6"/>
+      <c r="V6" s="1"/>
       <c r="W6" s="1"/>
       <c r="X6" s="1"/>
       <c r="Y6" s="1"/>
@@ -972,34 +937,33 @@
       <c r="AC6" s="1"/>
       <c r="AD6" s="1"/>
       <c r="AE6" s="1"/>
-      <c r="AF6" s="1"/>
-      <c r="AG6" s="9"/>
-      <c r="AH6" s="1"/>
-      <c r="AI6" s="9"/>
+      <c r="AF6" s="6"/>
+      <c r="AG6" s="1"/>
+      <c r="AH6" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="20.25">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="5"/>
       <c r="D7" s="1"/>
-      <c r="E7" s="3"/>
+      <c r="E7" s="10"/>
       <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="1"/>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="4"/>
-      <c r="Q7" s="1"/>
-      <c r="R7" s="9"/>
-      <c r="S7" s="9"/>
-      <c r="T7" s="1"/>
-      <c r="U7" s="9"/>
-      <c r="V7" s="9"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="1"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="1"/>
       <c r="W7" s="1"/>
       <c r="X7" s="1"/>
       <c r="Y7" s="1"/>
@@ -1009,34 +973,33 @@
       <c r="AC7" s="1"/>
       <c r="AD7" s="1"/>
       <c r="AE7" s="1"/>
-      <c r="AF7" s="1"/>
-      <c r="AG7" s="9"/>
-      <c r="AH7" s="1"/>
-      <c r="AI7" s="9"/>
+      <c r="AF7" s="6"/>
+      <c r="AG7" s="1"/>
+      <c r="AH7" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="20.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="5"/>
       <c r="D8" s="1"/>
-      <c r="E8" s="3"/>
+      <c r="E8" s="10"/>
       <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9"/>
-      <c r="O8" s="1"/>
-      <c r="P8" s="4"/>
-      <c r="Q8" s="1"/>
-      <c r="R8" s="9"/>
-      <c r="S8" s="9"/>
-      <c r="T8" s="1"/>
-      <c r="U8" s="9"/>
-      <c r="V8" s="9"/>
+      <c r="L8" s="6"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="6"/>
+      <c r="R8" s="6"/>
+      <c r="S8" s="1"/>
+      <c r="T8" s="6"/>
+      <c r="U8" s="6"/>
+      <c r="V8" s="1"/>
       <c r="W8" s="1"/>
       <c r="X8" s="1"/>
       <c r="Y8" s="1"/>
@@ -1046,10 +1009,9 @@
       <c r="AC8" s="1"/>
       <c r="AD8" s="1"/>
       <c r="AE8" s="1"/>
-      <c r="AF8" s="1"/>
-      <c r="AG8" s="9"/>
-      <c r="AH8" s="1"/>
-      <c r="AI8" s="9"/>
+      <c r="AF8" s="6"/>
+      <c r="AG8" s="1"/>
+      <c r="AH8" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>